<commit_message>
Apply review fixes to published content (Episode 1, templates, inventory note, README accuracy)
</commit_message>
<xml_diff>
--- a/templates/control-assessment.xlsx
+++ b/templates/control-assessment.xlsx
@@ -607,7 +607,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Examine, Interview</t>
+          <t>Examine and Interview</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Audit Record Review</t>
+          <t>Audit Record Review, Analysis, and Reporting</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>System Recovery</t>
+          <t>System Recovery and Reconstitution</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Identification and Authentication</t>
+          <t>Identification and Authentication (Organizational Users)</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Transmission Confidentiality</t>
+          <t>Transmission Confidentiality and Integrity</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Examine, Interview</t>
+          <t>Examine and Interview</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">

</xml_diff>